<commit_message>
FEM-5 builder: the section ends 5 m past the toe (26 m, was 44 m); a Voronoi variant of the toppling zone; the four workbooks rebuilt
The rock is elastic and both mechanisms are behind the face, so the 23 m of
ground past the toe did nothing but add elements. The toppling model's mesh
and solution sidecars are re-solved with the page's re-cut that follows.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_rock_joints.xlsx
+++ b/docs/tutorials/files/xslope_rock_joints.xlsx
@@ -12091,7 +12091,7 @@
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
-        <v>44.0</v>
+        <v>26.0</v>
       </c>
       <c r="B13" s="3">
         <v>0.0</v>
@@ -12135,7 +12135,7 @@
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
-        <v>44.0</v>
+        <v>26.0</v>
       </c>
       <c r="B14" s="3">
         <v>-3.0</v>

</xml_diff>